<commit_message>
Count Masters combat redesign: Y unification, swarm AI, multi-ring formation, boss prefab, pyramid victory
- Y position unified: PlayerPivot, SnowGirl_2, followers, enemies all at Y=0
- ObjectPooler moved under PlayerPivot as child
- Enemy formation: single ring -> multi-ring (SpawnMultiRingFormation)
- Enemy combat: WorldMover approach -> aggro -> individual swarm targeting nearest follower
- Separation physics: OverlapSphere 2m radius pushes enemies apart
- OnTriggerEnter instant clash: no pause/dash/coroutine/angle matching
- Boss: SnowmanSmall prefab (2x) instead of Capsule primitive, BossMinionController removed
- Victory staircase: 8877665544332211 pyramid, follower climbing, WorldMover freeze
- MoveFollower: Lerp removed -> instant position (leader+followers move as one unit)
- Excel: Boss rows (560/30/6, 550/50/8), Hole values set to 'left'
- Dead code cleanup: EnemyFormationController, BossMinionController deleted
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Levels/Levels.xlsx
+++ b/Assets/StreamingAssets/Levels/Levels.xlsx
@@ -6,14 +6,14 @@
     <workbookView tabRatio="600"/>
   </bookViews>
   <sheets>
-    <sheet name="Level1" sheetId="5" r:id="rId4"/>
-    <sheet name="Level2" sheetId="6" r:id="rId5"/>
+    <sheet name="Level1" sheetId="1" r:id="rId3"/>
+    <sheet name="Level2" sheetId="2" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="19">
   <si>
     <t xml:space="preserve">Distance</t>
   </si>
@@ -30,34 +30,22 @@
     <t xml:space="preserve">Gate</t>
   </si>
   <si>
-    <t xml:space="preserve">+5</t>
-  </si>
-  <si>
     <t xml:space="preserve">x2</t>
   </si>
   <si>
-    <t xml:space="preserve">+10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-3</t>
-  </si>
-  <si>
     <t xml:space="preserve">x3</t>
   </si>
   <si>
-    <t xml:space="preserve">+20</t>
-  </si>
-  <si>
     <t xml:space="preserve">Obstacle</t>
   </si>
   <si>
     <t xml:space="preserve">Saw</t>
   </si>
   <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+15</t>
+    <t xml:space="preserve">Hole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">left</t>
   </si>
   <si>
     <t xml:space="preserve">÷2</t>
@@ -69,49 +57,19 @@
     <t xml:space="preserve">Flame</t>
   </si>
   <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+30</t>
-  </si>
-  <si>
     <t xml:space="preserve">÷3</t>
   </si>
   <si>
-    <t xml:space="preserve">8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
     <t xml:space="preserve">x4</t>
   </si>
   <si>
-    <t xml:space="preserve">+100</t>
+    <t xml:space="preserve">Boss</t>
   </si>
   <si>
     <t xml:space="preserve">x5</t>
   </si>
   <si>
-    <t xml:space="preserve">12</t>
-  </si>
-  <si>
     <t xml:space="preserve">x10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+200</t>
   </si>
 </sst>
 </file>
@@ -154,9 +112,9 @@
 </styleSheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -180,11 +138,11 @@
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2">
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -194,11 +152,11 @@
       <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
+      <c r="C3">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <v>-3</v>
       </c>
     </row>
     <row r="4">
@@ -209,10 +167,10 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="D4">
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -220,167 +178,195 @@
         <v>110</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" t="s">
-        <v>13</v>
+        <v>8</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>170</v>
+        <v>130</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" t="s">
-        <v>17</v>
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="B8" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" t="s">
-        <v>6</v>
+        <v>13</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
+        <v>4</v>
+      </c>
+      <c r="C9">
+        <v>-10</v>
       </c>
       <c r="D9" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>270</v>
+        <v>240</v>
       </c>
       <c r="B10" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" t="s">
-        <v>21</v>
+        <v>8</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>310</v>
+        <v>270</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" t="s">
-        <v>17</v>
+        <v>4</v>
+      </c>
+      <c r="C11">
+        <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>350</v>
+        <v>310</v>
       </c>
       <c r="B12" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" t="s">
-        <v>23</v>
+        <v>13</v>
+      </c>
+      <c r="D12">
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>390</v>
+        <v>350</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s">
-        <v>13</v>
+        <v>5</v>
+      </c>
+      <c r="D13">
+        <v>50</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>430</v>
+        <v>390</v>
       </c>
       <c r="B14" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>24</v>
-      </c>
-      <c r="D14" t="s">
-        <v>25</v>
+        <v>8</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>470</v>
+        <v>430</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" t="s">
-        <v>17</v>
-      </c>
-      <c r="D15" t="s">
-        <v>26</v>
+        <v>4</v>
+      </c>
+      <c r="C15">
+        <v>25</v>
+      </c>
+      <c r="D15">
+        <v>-5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16">
+        <v>470</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
         <v>510</v>
       </c>
-      <c r="B16" t="s">
-        <v>4</v>
-      </c>
-      <c r="C16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" t="s">
-        <v>28</v>
+      <c r="B17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>560</v>
+      </c>
+      <c r="B18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18">
+        <v>30</v>
+      </c>
+      <c r="D18">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -388,9 +374,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -414,11 +400,11 @@
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
-        <v>7</v>
+      <c r="C2">
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -428,11 +414,11 @@
       <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" t="s">
-        <v>25</v>
+      <c r="C3">
+        <v>-5</v>
+      </c>
+      <c r="D3">
+        <v>-5</v>
       </c>
     </row>
     <row r="4">
@@ -440,167 +426,195 @@
         <v>90</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
+        <v>8</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>120</v>
+        <v>95</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" t="s">
-        <v>20</v>
+        <v>13</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" t="s">
-        <v>13</v>
+        <v>6</v>
+      </c>
+      <c r="D7">
+        <v>30</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" t="s">
-        <v>22</v>
+        <v>8</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>260</v>
+        <v>220</v>
       </c>
       <c r="B9" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" t="s">
-        <v>15</v>
+        <v>13</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>300</v>
+        <v>260</v>
       </c>
       <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10">
+        <v>50</v>
+      </c>
+      <c r="D10" t="s">
         <v>11</v>
-      </c>
-      <c r="C10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>340</v>
+        <v>300</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" t="s">
-        <v>26</v>
+        <v>8</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="B12" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" t="s">
-        <v>28</v>
+        <v>13</v>
+      </c>
+      <c r="D12">
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>420</v>
+        <v>380</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="D13">
+        <v>100</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>460</v>
+        <v>420</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" t="s">
-        <v>30</v>
+        <v>8</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15">
+        <v>460</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
         <v>500</v>
       </c>
-      <c r="B15" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" t="s">
-        <v>32</v>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>550</v>
+      </c>
+      <c r="B17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17">
+        <v>50</v>
+      </c>
+      <c r="D17">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: 디테일 계단 + Count Masters 장애물 (saw/wall/spinner) 구현
상세 계단 (detailed-stairs):
- Tread+Riser 3D 계단 구조, 사이드 레일, 개별 병력 블록, Crown 장식
- 계단 사이즈/폭/스텝수 조정, 점진적 피라미드 테이퍼
- Gold_Emission/Gold_Dark Material

Count Masters 장애물 (count-masters-obstacles):
- SawController: 회전 톱날 (Y축 2회전/초)
- Wall Barrier: 벽+틈 (left/right/center gap)
- SpinnerController: 회전 바 (Z축 90°/초)
- ObstacleType enum + SetObstacleType()
- AddObstacleTestData Editor 메뉴 (Tools/Add Obstacle Test Data)
- 도로 길이 증가 (+50→+80), 데이터 중복 방지

Etc:
- .gitignore 정리 (temp_xlsx.js, nul 제외)
- temp_xlsx.js 제거
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Levels/Levels.xlsx
+++ b/Assets/StreamingAssets/Levels/Levels.xlsx
@@ -1,35 +1,19 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes" xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
-  <ScaleCrop>false</ScaleCrop>
-  <LinksUpToDate>false</LinksUpToDate>
-  <SharedDoc>false</SharedDoc>
-  <HyperlinksChanged>false</HyperlinksChanged>
-  <Application>NPOI</Application>
-  <DocSecurity>0</DocSecurity>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr autoCompressPictures="1"/>
+  <bookViews>
+    <workbookView tabRatio="600"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Level1" sheetId="1" r:id="rId3"/>
+    <sheet name="Level2" sheetId="2" r:id="rId4"/>
+  </sheets>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties">
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-05-06T08:54:47Z</dcterms:created>
-  <dc:creator>NPOI</dc:creator>
-</coreProperties>
-</file>
-
-<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties">
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="2" name="Generator">
-    <lpwstr xmlns="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">NPOI</lpwstr>
-  </property>
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3" name="Generator Version">
-    <lpwstr xmlns="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">2.8.0</lpwstr>
-  </property>
-</Properties>
-</file>
-
-<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="29">
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="39">
   <si>
     <t xml:space="preserve">Distance</t>
   </si>
@@ -116,11 +100,41 @@
   </si>
   <si>
     <t xml:space="preserve">Finish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">obstacle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">saw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">left,1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spinner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">right,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">center,1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">left,2</t>
   </si>
 </sst>
 </file>
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
   <fonts count="1">
@@ -158,22 +172,9 @@
 </styleSheet>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr autoCompressPictures="1"/>
-  <bookViews>
-    <workbookView tabRatio="600"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Level1" sheetId="1" r:id="rId3"/>
-    <sheet name="Level2" sheetId="2" r:id="rId4"/>
-  </sheets>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -422,12 +423,152 @@
         <v>28</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>55</v>
+      </c>
+      <c r="B20" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" t="s">
+        <v>32</v>
+      </c>
+      <c r="D20" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>90</v>
+      </c>
+      <c r="B21" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>150</v>
+      </c>
+      <c r="B22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" t="s">
+        <v>32</v>
+      </c>
+      <c r="D22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>185</v>
+      </c>
+      <c r="B23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>260</v>
+      </c>
+      <c r="B24" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>330</v>
+      </c>
+      <c r="B25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" t="s">
+        <v>32</v>
+      </c>
+      <c r="D25" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>370</v>
+      </c>
+      <c r="B26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" t="s">
+        <v>30</v>
+      </c>
+      <c r="D26" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>450</v>
+      </c>
+      <c r="B27" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D27" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>490</v>
+      </c>
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" t="s">
+        <v>32</v>
+      </c>
+      <c r="D28" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>

</xml_diff>